<commit_message>
baseline dinamis data 2
</commit_message>
<xml_diff>
--- a/storage/app/Sumbu Grafik.xlsx
+++ b/storage/app/Sumbu Grafik.xlsx
@@ -897,16 +897,16 @@
         <v>OJA</v>
       </c>
       <c r="B30" t="str">
-        <v>1170</v>
+        <v>5400</v>
       </c>
       <c r="C30" t="str">
-        <v>2340</v>
+        <v>12600</v>
       </c>
       <c r="D30" t="str">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="E30" t="str">
-        <v>175</v>
+        <v>177</v>
       </c>
     </row>
     <row r="31">
@@ -914,16 +914,16 @@
         <v>ORU</v>
       </c>
       <c r="B31" t="str">
-        <v>1170</v>
+        <v>5400</v>
       </c>
       <c r="C31" t="str">
-        <v>2340</v>
+        <v>12600</v>
       </c>
       <c r="D31" t="str">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="E31" t="str">
-        <v>175</v>
+        <v>177</v>
       </c>
     </row>
     <row r="32">

</xml_diff>